<commit_message>
Add --indexing_method to PARSE
Added --indexing_method to PARSE/config.yaml to allow the user to define a start and end frame index instead of using times.

/tests/ was updated accordingly
</commit_message>
<xml_diff>
--- a/tests/trj/Example_AEM/Example_output_files/PSD_Plot.xlsx
+++ b/tests/trj/Example_AEM/Example_output_files/PSD_Plot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/42c400a6d2268350/Penn/GitHub/PARSE/tests/trj/Example_AEM/Example_output_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="115" documentId="8_{7149973D-7FBA-47E4-9186-8284705DD2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DF6B3EE-1FF8-4BE2-B210-3DDBF00B512B}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="8_{7149973D-7FBA-47E4-9186-8284705DD2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F858D45-624F-44D1-A43C-ADABBDA61119}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D12CB501-9D5F-4141-A117-3B2D7216ADD7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="6">
   <si>
     <t>Cumulaitve PSD</t>
   </si>
@@ -49,13 +49,27 @@
   <si>
     <t>d (A)</t>
   </si>
+  <si>
+    <t>PARSE, 1 frame</t>
+  </si>
+  <si>
+    <t>PARSE, 23 frames</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -85,7 +99,9 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -128,7 +144,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$C$1</c:f>
+              <c:f>Sheet1!$C$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -163,7 +179,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$31</c:f>
+              <c:f>Sheet1!$B$3:$B$32</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="30"/>
@@ -262,7 +278,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$C$2:$C$31</c:f>
+              <c:f>Sheet1!$C$3:$C$32</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="30"/>
@@ -385,7 +401,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$D$1</c:f>
+              <c:f>Sheet1!$D$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -420,7 +436,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$31</c:f>
+              <c:f>Sheet1!$B$3:$B$32</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="30"/>
@@ -519,7 +535,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$31</c:f>
+              <c:f>Sheet1!$D$3:$D$32</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="30"/>
@@ -1070,7 +1086,866 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>1 Frame</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$3:$B$32</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.315</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.33999999999999997</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.36499999999999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.39</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.41500000000000004</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.44000000000000006</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.46500000000000002</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.49000000000000005</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.51500000000000001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.54</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.56500000000000006</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.59000000000000008</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.61499999999999999</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.64</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.66500000000000004</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.69000000000000006</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.71500000000000008</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.74</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.76500000000000001</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.79</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.81500000000000006</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.84000000000000008</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.86499999999999999</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.89</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.91500000000000004</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.94000000000000006</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.96500000000000008</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.99</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1.0150000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$D$3:$D$32</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.0392000000000134</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.8539999999999894</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.5335999999999954</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.8571999999999953</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.4647999999999972</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.3152000000000048</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.3191999999999982</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.6176000000000024</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.2499999999999987</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.39199999999999963</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>9.0399999999999953E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.13600000000000048</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>6.8799999999999931E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.399999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>4.7999999999999952E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-970F-484B-B616-7963C120D03A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>23 Frames</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$3:$B$32</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.315</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.33999999999999997</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.36499999999999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.39</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.41500000000000004</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.44000000000000006</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.46500000000000002</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.49000000000000005</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.51500000000000001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.54</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.56500000000000006</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.59000000000000008</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.61499999999999999</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.64</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.66500000000000004</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.69000000000000006</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.71500000000000008</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.74</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.76500000000000001</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.79</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.81500000000000006</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.84000000000000008</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.86499999999999999</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.89</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.91500000000000004</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.94000000000000006</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.96500000000000008</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.99</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1.0150000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$I$3:$I$32</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.7116000000000113</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.2387999999999959</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.7159999999999913</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.2287999999999952</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.8151999999999973</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.5408000000000031</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.6483999999999983</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.0024000000000015</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.59439999999999937</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.26839999999999981</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.14959999999999987</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5.3600000000000189E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.5199999999999988E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.3599999999999989E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3.1999999999999976E-3</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-970F-484B-B616-7963C120D03A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="638607647"/>
+        <c:axId val="636349327"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="638607647"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>d (nm)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="636349327"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="636349327"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Pore Size Distribution</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="638607647"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1626,20 +2501,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>180974</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>238124</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>157161</xdr:rowOff>
+      <xdr:rowOff>52386</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>495299</xdr:colOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>552449</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>117156</xdr:rowOff>
+      <xdr:rowOff>12381</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1659,6 +3050,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>84364</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>89807</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>40</xdr:col>
+      <xdr:colOff>398689</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>49802</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA526672-B77F-4252-968D-40BFFFFFDD86}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1988,1021 +3417,956 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BA594D7-D524-4C7B-B376-D68CC69111AD}">
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
         <v>1</v>
       </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <f>A2/10</f>
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>3.15</v>
+        <v>0</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:B31" si="0">A3/10</f>
-        <v>0.315</v>
+        <f>A3/10</f>
+        <v>0</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <f>(C2-C3)/(B3-B2)</f>
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <f>F3/10</f>
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
+        <v>3.15</v>
+      </c>
+      <c r="B4">
+        <f t="shared" ref="B4:B32" si="0">A4/10</f>
+        <v>0.315</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <f>(C3-C4)/(B4-B3)</f>
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>3.15</v>
+      </c>
+      <c r="G4">
+        <f t="shared" ref="G4:G32" si="1">F4/10</f>
+        <v>0.315</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <f>(H3-H4)/(G4-G3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>3.4</v>
       </c>
-      <c r="B4">
+      <c r="B5">
         <f t="shared" si="0"/>
         <v>0.33999999999999997</v>
       </c>
-      <c r="C4">
+      <c r="C5">
         <v>0.79901999999999995</v>
       </c>
-      <c r="D4">
-        <f t="shared" ref="D4:D31" si="1">(C3-C4)/(B4-B3)</f>
+      <c r="D5">
+        <f t="shared" ref="D5:D32" si="2">(C4-C5)/(B5-B4)</f>
         <v>8.0392000000000134</v>
       </c>
+      <c r="F5">
+        <v>3.4</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="1"/>
+        <v>0.33999999999999997</v>
+      </c>
+      <c r="H5">
+        <v>0.75721000000000005</v>
+      </c>
+      <c r="I5">
+        <f t="shared" ref="I5:I32" si="3">(H4-H5)/(G5-G4)</f>
+        <v>9.7116000000000113</v>
+      </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>3.65</v>
       </c>
-      <c r="B5">
+      <c r="B6">
         <f t="shared" si="0"/>
         <v>0.36499999999999999</v>
       </c>
-      <c r="C5">
+      <c r="C6">
         <v>0.60267000000000004</v>
       </c>
-      <c r="D5">
+      <c r="D6">
+        <f t="shared" si="2"/>
+        <v>7.8539999999999894</v>
+      </c>
+      <c r="F6">
+        <v>3.65</v>
+      </c>
+      <c r="G6">
         <f t="shared" si="1"/>
-        <v>7.8539999999999894</v>
+        <v>0.36499999999999999</v>
+      </c>
+      <c r="H6">
+        <v>0.55123999999999995</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="3"/>
+        <v>8.2387999999999959</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>3.9</v>
       </c>
-      <c r="B6">
+      <c r="B7">
         <f t="shared" si="0"/>
         <v>0.39</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>0.43933</v>
       </c>
-      <c r="D6">
+      <c r="D7">
+        <f t="shared" si="2"/>
+        <v>6.5335999999999954</v>
+      </c>
+      <c r="F7">
+        <v>3.9</v>
+      </c>
+      <c r="G7">
         <f t="shared" si="1"/>
-        <v>6.5335999999999954</v>
+        <v>0.39</v>
+      </c>
+      <c r="H7">
+        <v>0.38334000000000001</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="3"/>
+        <v>6.7159999999999913</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>4.1500000000000004</v>
       </c>
-      <c r="B7">
+      <c r="B8">
         <f t="shared" si="0"/>
         <v>0.41500000000000004</v>
       </c>
-      <c r="C7">
+      <c r="C8">
         <v>0.31790000000000002</v>
       </c>
-      <c r="D7">
+      <c r="D8">
+        <f t="shared" si="2"/>
+        <v>4.8571999999999953</v>
+      </c>
+      <c r="F8">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="G8">
         <f t="shared" si="1"/>
-        <v>4.8571999999999953</v>
+        <v>0.41500000000000004</v>
+      </c>
+      <c r="H8">
+        <v>0.25262000000000001</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="3"/>
+        <v>5.2287999999999952</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>4.4000000000000004</v>
       </c>
-      <c r="B8">
+      <c r="B9">
         <f t="shared" si="0"/>
         <v>0.44000000000000006</v>
       </c>
-      <c r="C8">
+      <c r="C9">
         <v>0.23128000000000001</v>
       </c>
-      <c r="D8">
+      <c r="D9">
+        <f t="shared" si="2"/>
+        <v>3.4647999999999972</v>
+      </c>
+      <c r="F9">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="G9">
         <f t="shared" si="1"/>
-        <v>3.4647999999999972</v>
+        <v>0.44000000000000006</v>
+      </c>
+      <c r="H9">
+        <v>0.15723999999999999</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="3"/>
+        <v>3.8151999999999973</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>4.6500000000000004</v>
       </c>
-      <c r="B9">
+      <c r="B10">
         <f t="shared" si="0"/>
         <v>0.46500000000000002</v>
       </c>
-      <c r="C9">
+      <c r="C10">
         <v>0.1484</v>
       </c>
-      <c r="D9">
+      <c r="D10">
+        <f t="shared" si="2"/>
+        <v>3.3152000000000048</v>
+      </c>
+      <c r="F10">
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="G10">
         <f t="shared" si="1"/>
-        <v>3.3152000000000048</v>
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="H10">
+        <v>9.3719999999999998E-2</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="3"/>
+        <v>2.5408000000000031</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>4.9000000000000004</v>
       </c>
-      <c r="B10">
+      <c r="B11">
         <f t="shared" si="0"/>
         <v>0.49000000000000005</v>
       </c>
-      <c r="C10">
+      <c r="C11">
         <v>9.042E-2</v>
       </c>
-      <c r="D10">
+      <c r="D11">
+        <f t="shared" si="2"/>
+        <v>2.3191999999999982</v>
+      </c>
+      <c r="F11">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="G11">
         <f t="shared" si="1"/>
-        <v>2.3191999999999982</v>
+        <v>0.49000000000000005</v>
+      </c>
+      <c r="H11">
+        <v>5.2510000000000001E-2</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="3"/>
+        <v>1.6483999999999983</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>5.15</v>
       </c>
-      <c r="B11">
+      <c r="B12">
         <f t="shared" si="0"/>
         <v>0.51500000000000001</v>
       </c>
-      <c r="C11">
+      <c r="C12">
         <v>4.9979999999999997E-2</v>
       </c>
-      <c r="D11">
+      <c r="D12">
+        <f t="shared" si="2"/>
+        <v>1.6176000000000024</v>
+      </c>
+      <c r="F12">
+        <v>5.15</v>
+      </c>
+      <c r="G12">
         <f t="shared" si="1"/>
-        <v>1.6176000000000024</v>
+        <v>0.51500000000000001</v>
+      </c>
+      <c r="H12">
+        <v>2.7449999999999999E-2</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="3"/>
+        <v>1.0024000000000015</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>5.4</v>
       </c>
-      <c r="B12">
+      <c r="B13">
         <f t="shared" si="0"/>
         <v>0.54</v>
       </c>
-      <c r="C12">
+      <c r="C13">
         <v>1.873E-2</v>
       </c>
-      <c r="D12">
+      <c r="D13">
+        <f t="shared" si="2"/>
+        <v>1.2499999999999987</v>
+      </c>
+      <c r="F13">
+        <v>5.4</v>
+      </c>
+      <c r="G13">
         <f t="shared" si="1"/>
-        <v>1.2499999999999987</v>
+        <v>0.54</v>
+      </c>
+      <c r="H13">
+        <v>1.259E-2</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="3"/>
+        <v>0.59439999999999937</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>5.65</v>
       </c>
-      <c r="B13">
+      <c r="B14">
         <f t="shared" si="0"/>
         <v>0.56500000000000006</v>
       </c>
-      <c r="C13">
+      <c r="C14">
         <v>8.9300000000000004E-3</v>
       </c>
-      <c r="D13">
+      <c r="D14">
+        <f t="shared" si="2"/>
+        <v>0.39199999999999963</v>
+      </c>
+      <c r="F14">
+        <v>5.65</v>
+      </c>
+      <c r="G14">
         <f t="shared" si="1"/>
-        <v>0.39199999999999963</v>
+        <v>0.56500000000000006</v>
+      </c>
+      <c r="H14">
+        <v>5.8799999999999998E-3</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="3"/>
+        <v>0.26839999999999981</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>5.9</v>
       </c>
-      <c r="B14">
+      <c r="B15">
         <f t="shared" si="0"/>
         <v>0.59000000000000008</v>
       </c>
-      <c r="C14">
+      <c r="C15">
         <v>6.6699999999999997E-3</v>
       </c>
-      <c r="D14">
+      <c r="D15">
+        <f t="shared" si="2"/>
+        <v>9.0399999999999953E-2</v>
+      </c>
+      <c r="F15">
+        <v>5.9</v>
+      </c>
+      <c r="G15">
         <f t="shared" si="1"/>
-        <v>9.0399999999999953E-2</v>
+        <v>0.59000000000000008</v>
+      </c>
+      <c r="H15">
+        <v>2.14E-3</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="3"/>
+        <v>0.14959999999999987</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>6.15</v>
       </c>
-      <c r="B15">
+      <c r="B16">
         <f t="shared" si="0"/>
         <v>0.61499999999999999</v>
       </c>
-      <c r="C15">
+      <c r="C16">
         <v>3.2699999999999999E-3</v>
       </c>
-      <c r="D15">
+      <c r="D16">
+        <f t="shared" si="2"/>
+        <v>0.13600000000000048</v>
+      </c>
+      <c r="F16">
+        <v>6.15</v>
+      </c>
+      <c r="G16">
         <f t="shared" si="1"/>
-        <v>0.13600000000000048</v>
+        <v>0.61499999999999999</v>
+      </c>
+      <c r="H16">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="3"/>
+        <v>5.3600000000000189E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>6.4</v>
       </c>
-      <c r="B16">
+      <c r="B17">
         <f t="shared" si="0"/>
         <v>0.64</v>
       </c>
-      <c r="C16">
+      <c r="C17">
         <v>1.5499999999999999E-3</v>
       </c>
-      <c r="D16">
+      <c r="D17">
+        <f t="shared" si="2"/>
+        <v>6.8799999999999931E-2</v>
+      </c>
+      <c r="F17">
+        <v>6.4</v>
+      </c>
+      <c r="G17">
         <f t="shared" si="1"/>
-        <v>6.8799999999999931E-2</v>
+        <v>0.64</v>
+      </c>
+      <c r="H17">
+        <v>4.2000000000000002E-4</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="3"/>
+        <v>1.5199999999999988E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>6.65</v>
       </c>
-      <c r="B17">
+      <c r="B18">
         <f t="shared" si="0"/>
         <v>0.66500000000000004</v>
       </c>
-      <c r="C17">
+      <c r="C18">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="D17">
+      <c r="D18">
+        <f t="shared" si="2"/>
+        <v>1.399999999999999E-2</v>
+      </c>
+      <c r="F18">
+        <v>6.65</v>
+      </c>
+      <c r="G18">
         <f t="shared" si="1"/>
-        <v>1.399999999999999E-2</v>
+        <v>0.66500000000000004</v>
+      </c>
+      <c r="H18">
+        <v>8.0000000000000007E-5</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="3"/>
+        <v>1.3599999999999989E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>6.9</v>
       </c>
-      <c r="B18">
+      <c r="B19">
         <f t="shared" si="0"/>
         <v>0.69000000000000006</v>
       </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18">
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="2"/>
+        <v>4.7999999999999952E-2</v>
+      </c>
+      <c r="F19">
+        <v>6.9</v>
+      </c>
+      <c r="G19">
         <f t="shared" si="1"/>
-        <v>4.7999999999999952E-2</v>
+        <v>0.69000000000000006</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="3"/>
+        <v>3.1999999999999976E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>7.15</v>
       </c>
-      <c r="B19">
+      <c r="B20">
         <f t="shared" si="0"/>
         <v>0.71500000000000008</v>
       </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
-      <c r="D19">
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>7.15</v>
+      </c>
+      <c r="G20">
         <f t="shared" si="1"/>
+        <v>0.71500000000000008</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>7.4</v>
       </c>
-      <c r="B20">
+      <c r="B21">
         <f t="shared" si="0"/>
         <v>0.74</v>
       </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>7.4</v>
+      </c>
+      <c r="G21">
         <f t="shared" si="1"/>
+        <v>0.74</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>7.65</v>
       </c>
-      <c r="B21">
+      <c r="B22">
         <f t="shared" si="0"/>
         <v>0.76500000000000001</v>
       </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>7.65</v>
+      </c>
+      <c r="G22">
         <f t="shared" si="1"/>
+        <v>0.76500000000000001</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>7.9</v>
       </c>
-      <c r="B22">
+      <c r="B23">
         <f t="shared" si="0"/>
         <v>0.79</v>
       </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>7.9</v>
+      </c>
+      <c r="G23">
         <f t="shared" si="1"/>
+        <v>0.79</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>8.15</v>
       </c>
-      <c r="B23">
+      <c r="B24">
         <f t="shared" si="0"/>
         <v>0.81500000000000006</v>
       </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>8.15</v>
+      </c>
+      <c r="G24">
         <f t="shared" si="1"/>
+        <v>0.81500000000000006</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25">
         <v>8.4</v>
       </c>
-      <c r="B24">
+      <c r="B25">
         <f t="shared" si="0"/>
         <v>0.84000000000000008</v>
       </c>
-      <c r="C24">
-        <v>0</v>
-      </c>
-      <c r="D24">
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>8.4</v>
+      </c>
+      <c r="G25">
         <f t="shared" si="1"/>
+        <v>0.84000000000000008</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26">
         <v>8.65</v>
       </c>
-      <c r="B25">
+      <c r="B26">
         <f t="shared" si="0"/>
         <v>0.86499999999999999</v>
       </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
-      <c r="D25">
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>8.65</v>
+      </c>
+      <c r="G26">
         <f t="shared" si="1"/>
+        <v>0.86499999999999999</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27">
         <v>8.9</v>
       </c>
-      <c r="B26">
+      <c r="B27">
         <f t="shared" si="0"/>
         <v>0.89</v>
       </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26">
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>8.9</v>
+      </c>
+      <c r="G27">
         <f t="shared" si="1"/>
+        <v>0.89</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>9.15</v>
       </c>
-      <c r="B27">
+      <c r="B28">
         <f t="shared" si="0"/>
         <v>0.91500000000000004</v>
       </c>
-      <c r="C27">
-        <v>0</v>
-      </c>
-      <c r="D27">
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>9.15</v>
+      </c>
+      <c r="G28">
         <f t="shared" si="1"/>
+        <v>0.91500000000000004</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>9.4</v>
       </c>
-      <c r="B28">
+      <c r="B29">
         <f t="shared" si="0"/>
         <v>0.94000000000000006</v>
       </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="D28">
+      <c r="C29">
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>9.4</v>
+      </c>
+      <c r="G29">
         <f t="shared" si="1"/>
+        <v>0.94000000000000006</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30">
         <v>9.65</v>
       </c>
-      <c r="B29">
+      <c r="B30">
         <f t="shared" si="0"/>
         <v>0.96500000000000008</v>
       </c>
-      <c r="C29">
-        <v>0</v>
-      </c>
-      <c r="D29">
+      <c r="C30">
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>9.65</v>
+      </c>
+      <c r="G30">
         <f t="shared" si="1"/>
+        <v>0.96500000000000008</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31">
         <v>9.9</v>
       </c>
-      <c r="B30">
+      <c r="B31">
         <f t="shared" si="0"/>
         <v>0.99</v>
       </c>
-      <c r="C30">
-        <v>0</v>
-      </c>
-      <c r="D30">
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>9.9</v>
+      </c>
+      <c r="G31">
         <f t="shared" si="1"/>
+        <v>0.99</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32">
         <v>10.15</v>
       </c>
-      <c r="B31">
+      <c r="B32">
         <f t="shared" si="0"/>
         <v>1.0150000000000001</v>
       </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
-      <c r="D31">
+      <c r="C32">
+        <v>0</v>
+      </c>
+      <c r="D32">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>10.15</v>
+      </c>
+      <c r="G32">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H31" s="1"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H32" s="1"/>
-    </row>
-    <row r="33" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H33" s="1"/>
-    </row>
-    <row r="34" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G34">
-        <f>3.9/2</f>
-        <v>1.95</v>
-      </c>
-      <c r="H34" s="1"/>
-    </row>
-    <row r="35" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H35" s="1"/>
-    </row>
-    <row r="36" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H36" s="1"/>
-    </row>
-    <row r="37" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H37" s="1"/>
-    </row>
-    <row r="38" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H38" s="1"/>
-    </row>
-    <row r="39" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H39" s="1"/>
-    </row>
-    <row r="40" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H40" s="1"/>
-    </row>
-    <row r="41" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H41" s="1"/>
-    </row>
-    <row r="42" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H42" s="1"/>
-    </row>
-    <row r="43" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H43" s="1"/>
-    </row>
-    <row r="44" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H44" s="1"/>
-    </row>
-    <row r="45" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H45" s="1"/>
-    </row>
-    <row r="46" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H46" s="1"/>
-    </row>
-    <row r="47" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H47" s="1"/>
-    </row>
-    <row r="48" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="H48" s="1"/>
-    </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H49" s="1"/>
-    </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H50" s="1"/>
-    </row>
-    <row r="51" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H51" s="1"/>
-    </row>
-    <row r="52" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H52" s="1"/>
-    </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H53" s="1"/>
-    </row>
-    <row r="54" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H54" s="1"/>
-    </row>
-    <row r="55" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H55" s="1"/>
-    </row>
-    <row r="56" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H56" s="1"/>
-    </row>
-    <row r="57" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H57" s="1"/>
-    </row>
-    <row r="58" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H58" s="1"/>
-    </row>
-    <row r="59" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H59" s="1"/>
-    </row>
-    <row r="60" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H60" s="1"/>
-    </row>
-    <row r="61" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H61" s="1"/>
-    </row>
-    <row r="62" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H62" s="1"/>
-    </row>
-    <row r="63" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H63" s="1"/>
-    </row>
-    <row r="64" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H64" s="1"/>
-    </row>
-    <row r="65" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H65" s="1"/>
-    </row>
-    <row r="66" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H66" s="1"/>
-    </row>
-    <row r="67" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H67" s="1"/>
-    </row>
-    <row r="68" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H68" s="1"/>
-    </row>
-    <row r="69" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H69" s="1"/>
-    </row>
-    <row r="70" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H70" s="1"/>
-    </row>
-    <row r="71" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H71" s="1"/>
-    </row>
-    <row r="72" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H72" s="1"/>
-    </row>
-    <row r="73" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H73" s="1"/>
-    </row>
-    <row r="74" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H74" s="1"/>
-    </row>
-    <row r="75" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H75" s="1"/>
-    </row>
-    <row r="76" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H76" s="1"/>
-    </row>
-    <row r="77" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H77" s="1"/>
-    </row>
-    <row r="78" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H78" s="1"/>
-    </row>
-    <row r="79" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H79" s="1"/>
-    </row>
-    <row r="80" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H80" s="1"/>
-    </row>
-    <row r="81" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H81" s="1"/>
-    </row>
-    <row r="82" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H82" s="1"/>
-    </row>
-    <row r="83" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H83" s="1"/>
-    </row>
-    <row r="84" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H84" s="1"/>
-    </row>
-    <row r="85" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H85" s="1"/>
-    </row>
-    <row r="86" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H86" s="1"/>
-    </row>
-    <row r="87" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H87" s="1"/>
-    </row>
-    <row r="88" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H88" s="1"/>
-    </row>
-    <row r="89" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H89" s="1"/>
-    </row>
-    <row r="90" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H90" s="1"/>
-    </row>
-    <row r="91" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H91" s="1"/>
-    </row>
-    <row r="92" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H92" s="1"/>
-    </row>
-    <row r="93" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H93" s="1"/>
-    </row>
-    <row r="94" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H94" s="1"/>
-    </row>
-    <row r="95" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H95" s="1"/>
-    </row>
-    <row r="96" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H96" s="1"/>
-    </row>
-    <row r="97" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H97" s="1"/>
-    </row>
-    <row r="98" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H98" s="1"/>
-    </row>
-    <row r="99" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H99" s="1"/>
-    </row>
-    <row r="100" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H100" s="1"/>
-    </row>
-    <row r="101" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H101" s="1"/>
-    </row>
-    <row r="102" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H102" s="1"/>
-    </row>
-    <row r="103" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H103" s="1"/>
-    </row>
-    <row r="104" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H104" s="1"/>
-    </row>
-    <row r="105" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H105" s="1"/>
-    </row>
-    <row r="106" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H106" s="1"/>
-    </row>
-    <row r="107" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H107" s="1"/>
-    </row>
-    <row r="108" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H108" s="1"/>
-    </row>
-    <row r="109" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H109" s="1"/>
-    </row>
-    <row r="110" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H110" s="1"/>
-    </row>
-    <row r="111" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H111" s="1"/>
-    </row>
-    <row r="112" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H112" s="1"/>
-    </row>
-    <row r="113" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H113" s="1"/>
-    </row>
-    <row r="114" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H114" s="1"/>
-    </row>
-    <row r="115" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H115" s="1"/>
-    </row>
-    <row r="116" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H116" s="1"/>
-    </row>
-    <row r="117" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H117" s="1"/>
-    </row>
-    <row r="118" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H118" s="1"/>
-    </row>
-    <row r="119" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H119" s="1"/>
-    </row>
-    <row r="120" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H120" s="1"/>
-    </row>
-    <row r="121" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H121" s="1"/>
-    </row>
-    <row r="122" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H122" s="1"/>
-    </row>
-    <row r="123" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H123" s="1"/>
-    </row>
-    <row r="124" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H124" s="1"/>
-    </row>
-    <row r="125" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H125" s="1"/>
-    </row>
-    <row r="126" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H126" s="1"/>
-    </row>
-    <row r="127" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H127" s="1"/>
-    </row>
-    <row r="128" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H128" s="1"/>
-    </row>
-    <row r="129" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H129" s="1"/>
-    </row>
-    <row r="130" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H130" s="1"/>
-    </row>
-    <row r="131" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H131" s="1"/>
-    </row>
-    <row r="132" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H132" s="1"/>
-    </row>
-    <row r="133" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H133" s="1"/>
-    </row>
-    <row r="134" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H134" s="1"/>
-    </row>
-    <row r="135" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H135" s="1"/>
-    </row>
-    <row r="136" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H136" s="1"/>
-    </row>
-    <row r="137" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H137" s="1"/>
-    </row>
-    <row r="138" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H138" s="1"/>
-    </row>
-    <row r="139" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H139" s="1"/>
-    </row>
-    <row r="140" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H140" s="1"/>
-    </row>
-    <row r="141" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H141" s="1"/>
-    </row>
-    <row r="142" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H142" s="1"/>
-    </row>
-    <row r="143" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H143" s="1"/>
-    </row>
-    <row r="144" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H144" s="1"/>
-    </row>
-    <row r="145" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H145" s="1"/>
-    </row>
-    <row r="146" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H146" s="1"/>
-    </row>
-    <row r="147" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H147" s="1"/>
-    </row>
-    <row r="148" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H148" s="1"/>
-    </row>
-    <row r="149" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H149" s="1"/>
-    </row>
-    <row r="150" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H150" s="1"/>
-    </row>
-    <row r="151" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H151" s="1"/>
-    </row>
-    <row r="152" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H152" s="1"/>
-    </row>
-    <row r="153" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H153" s="1"/>
-    </row>
-    <row r="154" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H154" s="1"/>
-    </row>
-    <row r="155" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H155" s="1"/>
-    </row>
-    <row r="156" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H156" s="1"/>
-    </row>
-    <row r="157" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H157" s="1"/>
-    </row>
-    <row r="158" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H158" s="1"/>
-    </row>
-    <row r="159" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H159" s="1"/>
-    </row>
-    <row r="160" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H160" s="1"/>
-    </row>
-    <row r="161" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H161" s="1"/>
-    </row>
-    <row r="162" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H162" s="1"/>
-    </row>
-    <row r="163" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H163" s="1"/>
-    </row>
-    <row r="164" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H164" s="1"/>
-    </row>
-    <row r="165" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H165" s="1"/>
-    </row>
-    <row r="166" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H166" s="1"/>
-    </row>
-    <row r="167" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H167" s="1"/>
-    </row>
-    <row r="168" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H168" s="1"/>
-    </row>
-    <row r="169" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H169" s="1"/>
-    </row>
-    <row r="170" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H170" s="1"/>
-    </row>
-    <row r="171" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H171" s="1"/>
-    </row>
-    <row r="172" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H172" s="1"/>
-    </row>
-    <row r="173" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H173" s="1"/>
-    </row>
-    <row r="174" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H174" s="1"/>
-    </row>
-    <row r="175" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H175" s="1"/>
-    </row>
-    <row r="176" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H176" s="1"/>
-    </row>
-    <row r="177" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H177" s="1"/>
-    </row>
-    <row r="178" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H178" s="1"/>
-    </row>
-    <row r="179" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H179" s="1"/>
-    </row>
-    <row r="180" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H180" s="1"/>
-    </row>
-    <row r="181" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H181" s="1"/>
-    </row>
-    <row r="182" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H182" s="1"/>
-    </row>
-    <row r="183" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H183" s="1"/>
-    </row>
-    <row r="184" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H184" s="1"/>
-    </row>
-    <row r="185" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H185" s="1"/>
-    </row>
-    <row r="186" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H186" s="1"/>
-    </row>
-    <row r="187" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H187" s="1"/>
-    </row>
-    <row r="188" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H188" s="1"/>
-    </row>
-    <row r="189" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H189" s="1"/>
-    </row>
-    <row r="190" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H190" s="1"/>
-    </row>
-    <row r="191" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H191" s="1"/>
-    </row>
-    <row r="192" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H192" s="1"/>
-    </row>
-    <row r="193" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H193" s="1"/>
-    </row>
-    <row r="194" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H194" s="1"/>
-    </row>
-    <row r="195" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H195" s="1"/>
-    </row>
-    <row r="196" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H196" s="1"/>
-    </row>
-    <row r="197" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H197" s="1"/>
-    </row>
-    <row r="198" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H198" s="1"/>
-    </row>
-    <row r="199" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H199" s="1"/>
-    </row>
-    <row r="200" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H200" s="1"/>
-    </row>
-    <row r="201" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H201" s="1"/>
+        <v>1.0150000000000001</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="F1:I1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>